<commit_message>
feat: adiciona dashboard Ativuz, README e resolve conflito no .gitignore
- Resolve conflito de merge no .gitignore (mescla templates Next.js e Python/Flask)
- Adiciona arquivos do Ativuz Dashboard (HTML, CSS, componentes JSX, assets)
- Atualiza planilha CONTAS-A-RECEBER.xlsx
- Adiciona README.md e prompt_lovable_ativuz.md

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docx_templates/CONTAS-A-RECEBER.xlsx
+++ b/docx_templates/CONTAS-A-RECEBER.xlsx
@@ -9,14 +9,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Relatório!$A$5:$S$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Relatório!$A$1:$S$68</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Relatório!$A$1:$S$65</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1" fullPrecision="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="130">
   <si>
     <t>Contas a Receber em aberto</t>
   </si>
@@ -36,11 +36,11 @@
         <color rgb="FF808080"/>
         <sz val="11"/>
       </rPr>
-      <t>Data Final: 30/04/2026, Conta de Recebimento: 1.0 [OFICIAL] SICREDI | BANCO GESTOR</t>
+      <t>Data Inicial: 01/08/2025, Data Final: 30/04/2026, Conta de Recebimento: 1.0 [OFICIAL] SICREDI | BANCO GESTOR</t>
     </r>
   </si>
   <si>
-    <t>Relatório exportado em segunda-feira, 27 de abril de 2026 por KAROL MEDEIROS</t>
+    <t>Relatório exportado em terça-feira, 28 de abril de 2026 por KAROL MEDEIROS</t>
   </si>
   <si>
     <t>Conta de Recebimento</t>
@@ -142,70 +142,127 @@
     <t>AZ EMPREENDIMENTOS</t>
   </si>
   <si>
-    <t>FA-11447</t>
+    <t>FA-11421</t>
+  </si>
+  <si>
+    <t>FA-11255</t>
+  </si>
+  <si>
+    <t>LEONARDO GOMES DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11406</t>
+  </si>
+  <si>
+    <t>DAVI HENRIQUE DANTAS DE SOUZA</t>
+  </si>
+  <si>
+    <t>FA-11383</t>
+  </si>
+  <si>
+    <t>JOZILDO TARQUINO DE BRITO</t>
+  </si>
+  <si>
+    <t>FA-11419</t>
+  </si>
+  <si>
+    <t>YURI BATISTA DA COSTA</t>
+  </si>
+  <si>
+    <t>LUCAS SANTOS REVOREDO DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11182</t>
+  </si>
+  <si>
+    <t>MARCELO BENTO DE ARAUJO</t>
+  </si>
+  <si>
+    <t>FA-11069</t>
+  </si>
+  <si>
+    <t>ALBERTO MANOEL DOS REIS</t>
+  </si>
+  <si>
+    <t>PRIVADO</t>
+  </si>
+  <si>
+    <t>ND-11305</t>
+  </si>
+  <si>
+    <t>NOTA DE DÉBITO</t>
+  </si>
+  <si>
+    <t>FA-11455</t>
+  </si>
+  <si>
+    <t>RAFAEL CAVALCANTI BARROS FERREIRA</t>
+  </si>
+  <si>
+    <t>FA-11426</t>
+  </si>
+  <si>
+    <t>FA-11244</t>
+  </si>
+  <si>
+    <t>FA-11115</t>
+  </si>
+  <si>
+    <t>NICOLAS JUAN HENRIQUE SILVA DE MARIA</t>
+  </si>
+  <si>
+    <t>FA-11453</t>
   </si>
   <si>
     <t>DERICK PEDRO BEZERRA DA ROCHA</t>
   </si>
   <si>
-    <t>FA-11421</t>
-  </si>
-  <si>
-    <t>FA-11255</t>
-  </si>
-  <si>
-    <t>LEONARDO GOMES DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>FA-11406</t>
-  </si>
-  <si>
-    <t>DAVI HENRIQUE DANTAS DE SOUZA</t>
-  </si>
-  <si>
-    <t>FA-11383</t>
-  </si>
-  <si>
-    <t>JOZILDO TARQUINO DE BRITO</t>
-  </si>
-  <si>
-    <t>FA-11419</t>
-  </si>
-  <si>
-    <t>YURI BATISTA DA COSTA</t>
-  </si>
-  <si>
-    <t>LUCAS SANTOS REVOREDO DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>FA-11189</t>
-  </si>
-  <si>
-    <t>FA-11182</t>
-  </si>
-  <si>
-    <t>MARCELO BENTO DE ARAUJO</t>
-  </si>
-  <si>
-    <t>FA-11069</t>
-  </si>
-  <si>
-    <t>ALBERTO MANOEL DOS REIS</t>
-  </si>
-  <si>
-    <t>PRIVADO</t>
-  </si>
-  <si>
-    <t>ND-11305</t>
-  </si>
-  <si>
-    <t>NOTA DE DÉBITO</t>
+    <t>FA-11424</t>
+  </si>
+  <si>
+    <t>FA-11407</t>
+  </si>
+  <si>
+    <t>FA-11256</t>
+  </si>
+  <si>
+    <t>FA-11183</t>
+  </si>
+  <si>
+    <t>FA-11361</t>
+  </si>
+  <si>
+    <t>RAMON TALLES BARBALHO DE FRANÇA</t>
+  </si>
+  <si>
+    <t>FA-11452</t>
+  </si>
+  <si>
+    <t>YAGO ELIAS COSTA BATISTA</t>
+  </si>
+  <si>
+    <t>FA-11114</t>
+  </si>
+  <si>
+    <t>FA-11456</t>
+  </si>
+  <si>
+    <t>FERNANDO RODRIGUES DO NASCIMENTO</t>
   </si>
   <si>
     <t>FA-11113</t>
   </si>
   <si>
-    <t>NICOLAS JUAN HENRIQUE SILVA DE MARIA</t>
+    <t>FA-11253</t>
+  </si>
+  <si>
+    <t>FA-11387</t>
+  </si>
+  <si>
+    <t>ADRIANO SANTOS DE CARVALHO</t>
+  </si>
+  <si>
+    <t>FA-11147</t>
   </si>
   <si>
     <t>VENCIDO ACIMA DE 90 DIAS</t>
@@ -217,220 +274,154 @@
     <t>RICARDO ARAUJO DE MIRANDA</t>
   </si>
   <si>
-    <t>FA-11455</t>
-  </si>
-  <si>
-    <t>RAFAEL CAVALCANTI BARROS FERREIRA</t>
-  </si>
-  <si>
-    <t>FA-11426</t>
-  </si>
-  <si>
-    <t>FA-11244</t>
-  </si>
-  <si>
     <t>FA-11390</t>
   </si>
   <si>
-    <t>ADRIANO SANTOS DE CARVALHO</t>
-  </si>
-  <si>
-    <t>FA-11453</t>
-  </si>
-  <si>
-    <t>FA-11115</t>
-  </si>
-  <si>
-    <t>FA-11256</t>
-  </si>
-  <si>
-    <t>FA-11424</t>
-  </si>
-  <si>
-    <t>FA-11407</t>
-  </si>
-  <si>
-    <t>FA-11183</t>
-  </si>
-  <si>
-    <t>FA-11361</t>
-  </si>
-  <si>
-    <t>RAMON TALLES BARBALHO DE FRANÇA</t>
-  </si>
-  <si>
-    <t>FA-11452</t>
-  </si>
-  <si>
-    <t>YAGO ELIAS COSTA BATISTA</t>
-  </si>
-  <si>
-    <t>FA-11346</t>
-  </si>
-  <si>
-    <t>FA-11114</t>
-  </si>
-  <si>
-    <t>FA-11456</t>
-  </si>
-  <si>
-    <t>FERNANDO RODRIGUES DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>FA-11253</t>
-  </si>
-  <si>
-    <t>FA-11387</t>
+    <t>FA-11516</t>
+  </si>
+  <si>
+    <t>ROBERTO MURATORI</t>
+  </si>
+  <si>
+    <t>FA-11458</t>
+  </si>
+  <si>
+    <t>FA-11392</t>
+  </si>
+  <si>
+    <t>FA-11153</t>
+  </si>
+  <si>
+    <t>FA-11462</t>
+  </si>
+  <si>
+    <t>FA-11517</t>
+  </si>
+  <si>
+    <t>JONILSON JOSEMAR DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11351</t>
+  </si>
+  <si>
+    <t>MARIO EWERTON CANDIDO DE SOUZA</t>
+  </si>
+  <si>
+    <t>FA-11350</t>
+  </si>
+  <si>
+    <t>FA-11393</t>
+  </si>
+  <si>
+    <t>FA-11391</t>
+  </si>
+  <si>
+    <t>ANA FLORIPES CARVALHO DA CUNHA</t>
+  </si>
+  <si>
+    <t>FA-11485</t>
+  </si>
+  <si>
+    <t>ROSSILY PEREIRA DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11460</t>
+  </si>
+  <si>
+    <t>FA-11111</t>
+  </si>
+  <si>
+    <t>FA-11369</t>
+  </si>
+  <si>
+    <t>PEDRO GABRIEL FASANARO DE OLIVEIRA</t>
+  </si>
+  <si>
+    <t>FA-11500</t>
+  </si>
+  <si>
+    <t>WESCLY JEAN DE MEDEIROS</t>
+  </si>
+  <si>
+    <t>FA-11497</t>
+  </si>
+  <si>
+    <t>FA-11430</t>
+  </si>
+  <si>
+    <t>RAYANE ROBERTA DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11463</t>
+  </si>
+  <si>
+    <t>LUCAS NAJA MOURA RODRIGUES</t>
+  </si>
+  <si>
+    <t>FA-11408</t>
+  </si>
+  <si>
+    <t>FA-11352</t>
+  </si>
+  <si>
+    <t>ANDERSON QUEIROZ PINHEIRO</t>
+  </si>
+  <si>
+    <t>FA-11518</t>
+  </si>
+  <si>
+    <t>FA-11459</t>
+  </si>
+  <si>
+    <t>FA-11325</t>
+  </si>
+  <si>
+    <t>MAICON LOPES SILVA</t>
+  </si>
+  <si>
+    <t>FA-11265</t>
+  </si>
+  <si>
+    <t>ANNY KATARINA ACIOLE DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11461</t>
+  </si>
+  <si>
+    <t>FA-11545</t>
+  </si>
+  <si>
+    <t>REGINALDO BENTO DA SILVA</t>
+  </si>
+  <si>
+    <t>JOÃO PAULO CONSÓRCIOS</t>
+  </si>
+  <si>
+    <t>FA-11348</t>
   </si>
   <si>
     <t>HOJE</t>
   </si>
   <si>
-    <t>FA-11147</t>
-  </si>
-  <si>
-    <t>FA-11458</t>
-  </si>
-  <si>
-    <t>FA-11392</t>
-  </si>
-  <si>
-    <t>FA-11516</t>
-  </si>
-  <si>
-    <t>ROBERTO MURATORI</t>
-  </si>
-  <si>
-    <t>FA-11462</t>
-  </si>
-  <si>
-    <t>FA-11153</t>
-  </si>
-  <si>
-    <t>FA-11393</t>
-  </si>
-  <si>
-    <t>FA-11351</t>
-  </si>
-  <si>
-    <t>MARIO EWERTON CANDIDO DE SOUZA</t>
-  </si>
-  <si>
-    <t>FA-11350</t>
-  </si>
-  <si>
-    <t>FA-11391</t>
-  </si>
-  <si>
-    <t>ANA FLORIPES CARVALHO DA CUNHA</t>
-  </si>
-  <si>
-    <t>FA-11485</t>
-  </si>
-  <si>
-    <t>ROSSILY PEREIRA DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11517</t>
-  </si>
-  <si>
-    <t>JONILSON JOSEMAR DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>FA-11500</t>
-  </si>
-  <si>
-    <t>WESCLY JEAN DE MEDEIROS</t>
-  </si>
-  <si>
-    <t>FA-11497</t>
-  </si>
-  <si>
-    <t>FA-11460</t>
-  </si>
-  <si>
-    <t>FA-11369</t>
-  </si>
-  <si>
-    <t>PEDRO GABRIEL FASANARO DE OLIVEIRA</t>
-  </si>
-  <si>
-    <t>FA-11111</t>
-  </si>
-  <si>
     <t>FA-11276</t>
   </si>
   <si>
     <t>FELIPE DA SILVA</t>
   </si>
   <si>
-    <t>FA-11430</t>
-  </si>
-  <si>
-    <t>RAYANE ROBERTA DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11463</t>
-  </si>
-  <si>
-    <t>LUCAS NAJA MOURA RODRIGUES</t>
-  </si>
-  <si>
-    <t>FA-11408</t>
-  </si>
-  <si>
-    <t>FA-11352</t>
-  </si>
-  <si>
-    <t>ANDERSON QUEIROZ PINHEIRO</t>
-  </si>
-  <si>
-    <t>FA-11459</t>
-  </si>
-  <si>
-    <t>FA-11518</t>
-  </si>
-  <si>
-    <t>FA-11325</t>
-  </si>
-  <si>
-    <t>MAICON LOPES SILVA</t>
-  </si>
-  <si>
-    <t>FA-11265</t>
-  </si>
-  <si>
-    <t>ANNY KATARINA ACIOLE DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11461</t>
-  </si>
-  <si>
-    <t>FA-11545</t>
-  </si>
-  <si>
-    <t>REGINALDO BENTO DA SILVA</t>
-  </si>
-  <si>
-    <t>JOÃO PAULO CONSÓRCIOS</t>
-  </si>
-  <si>
-    <t>FA-11348</t>
+    <t>FA-11347</t>
+  </si>
+  <si>
+    <t>FA-11446</t>
+  </si>
+  <si>
+    <t>FA-11362</t>
+  </si>
+  <si>
+    <t>ANA CONCEIÇÃO CARNEIRO DE ALBUQUERQUE</t>
   </si>
   <si>
     <t>A VENCER</t>
-  </si>
-  <si>
-    <t>FA-11347</t>
-  </si>
-  <si>
-    <t>FA-11446</t>
-  </si>
-  <si>
-    <t>FA-11362</t>
-  </si>
-  <si>
-    <t>ANA CONCEIÇÃO CARNEIRO DE ALBUQUERQUE</t>
   </si>
 </sst>
 </file>
@@ -573,7 +564,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName=""/>
-  <dimension ref="A1:S74"/>
+  <dimension ref="A1:S71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="38.13657760620117" customWidth="1" style="1"/>
@@ -690,10 +681,10 @@
         <v>46086</v>
       </c>
       <c r="F6" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="G6" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>23</v>
@@ -749,10 +740,10 @@
         <v>25</v>
       </c>
       <c r="F7" s="8">
-        <v>-35</v>
+        <v>-36</v>
       </c>
       <c r="G7" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>30</v>
@@ -808,10 +799,10 @@
         <v>46122</v>
       </c>
       <c r="F8" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="G8" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="H8" s="6" t="s">
         <v>23</v>
@@ -864,13 +855,13 @@
         <v>46125</v>
       </c>
       <c r="E9" s="7">
-        <v>46119</v>
+        <v>46118</v>
       </c>
       <c r="F9" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="G9" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>23</v>
@@ -885,10 +876,10 @@
         <v>25</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="N9" s="6" t="s">
         <v>27</v>
@@ -906,7 +897,7 @@
         <v>29</v>
       </c>
       <c r="S9" s="9">
-        <v>650</v>
+        <v>680</v>
       </c>
     </row>
     <row r="10" ht="23" customHeight="1">
@@ -923,13 +914,13 @@
         <v>46125</v>
       </c>
       <c r="E10" s="7">
-        <v>46118</v>
+        <v>46087</v>
       </c>
       <c r="F10" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="G10" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>23</v>
@@ -938,13 +929,13 @@
         <v>23</v>
       </c>
       <c r="J10" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L10" s="6" t="s">
         <v>38</v>
-      </c>
-      <c r="K10" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L10" s="6" t="s">
-        <v>32</v>
       </c>
       <c r="M10" s="6" t="s">
         <v>25</v>
@@ -982,13 +973,13 @@
         <v>46125</v>
       </c>
       <c r="E11" s="7">
-        <v>46087</v>
+        <v>46113</v>
       </c>
       <c r="F11" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="G11" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>23</v>
@@ -1006,7 +997,7 @@
         <v>40</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="N11" s="6" t="s">
         <v>27</v>
@@ -1032,19 +1023,19 @@
         <v>22</v>
       </c>
       <c r="B12" s="7">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="C12" s="7">
-        <v>46125</v>
+        <v>46118</v>
       </c>
       <c r="D12" s="7">
-        <v>46125</v>
-      </c>
-      <c r="E12" s="7">
-        <v>46113</v>
+        <v>46118</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F12" s="8">
-        <v>-14</v>
+        <v>-22</v>
       </c>
       <c r="G12" s="8">
         <v>-14</v>
@@ -1077,13 +1068,13 @@
         <v>25</v>
       </c>
       <c r="Q12" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="R12" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S12" s="9">
-        <v>680</v>
+        <v>130.16</v>
       </c>
     </row>
     <row r="13" ht="23" customHeight="1">
@@ -1103,10 +1094,10 @@
         <v>25</v>
       </c>
       <c r="F13" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="G13" s="8">
-        <v>-13</v>
+        <v>-14</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>23</v>
@@ -1124,7 +1115,7 @@
         <v>44</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="N13" s="6" t="s">
         <v>27</v>
@@ -1142,7 +1133,7 @@
         <v>29</v>
       </c>
       <c r="S13" s="9">
-        <v>130.16</v>
+        <v>400</v>
       </c>
     </row>
     <row r="14" ht="23" customHeight="1">
@@ -1150,7 +1141,7 @@
         <v>22</v>
       </c>
       <c r="B14" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="C14" s="7">
         <v>46118</v>
@@ -1162,7 +1153,7 @@
         <v>25</v>
       </c>
       <c r="F14" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="G14" s="8">
         <v>-13</v>
@@ -1174,14 +1165,14 @@
         <v>23</v>
       </c>
       <c r="J14" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L14" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="K14" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L14" s="6" t="s">
-        <v>46</v>
-      </c>
       <c r="M14" s="6" t="s">
         <v>25</v>
       </c>
@@ -1201,7 +1192,7 @@
         <v>29</v>
       </c>
       <c r="S14" s="9">
-        <v>400</v>
+        <v>260</v>
       </c>
     </row>
     <row r="15" ht="23" customHeight="1">
@@ -1209,31 +1200,31 @@
         <v>22</v>
       </c>
       <c r="B15" s="7">
-        <v>46127</v>
+        <v>46129</v>
       </c>
       <c r="C15" s="7">
-        <v>46118</v>
+        <v>46104</v>
       </c>
       <c r="D15" s="7">
-        <v>46118</v>
+        <v>46104</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F15" s="8">
-        <v>-21</v>
+        <v>-36</v>
       </c>
       <c r="G15" s="8">
-        <v>-12</v>
+        <v>-11</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="I15" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="K15" s="6" t="s">
         <v>25</v>
@@ -1257,10 +1248,10 @@
         <v>25</v>
       </c>
       <c r="R15" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="S15" s="9">
-        <v>260</v>
+        <v>357.49</v>
       </c>
     </row>
     <row r="16" ht="23" customHeight="1">
@@ -1268,22 +1259,22 @@
         <v>22</v>
       </c>
       <c r="B16" s="7">
-        <v>46128</v>
+        <v>46132</v>
       </c>
       <c r="C16" s="7">
-        <v>46111</v>
+        <v>46118</v>
       </c>
       <c r="D16" s="7">
-        <v>46111</v>
+        <v>46118</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F16" s="8">
-        <v>-28</v>
+        <v>-22</v>
       </c>
       <c r="G16" s="8">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>23</v>
@@ -1298,10 +1289,10 @@
         <v>25</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="M16" s="6" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="N16" s="6" t="s">
         <v>27</v>
@@ -1310,7 +1301,7 @@
         <v>27</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="Q16" s="6" t="s">
         <v>25</v>
@@ -1319,7 +1310,7 @@
         <v>29</v>
       </c>
       <c r="S16" s="9">
-        <v>119.57</v>
+        <v>91.54</v>
       </c>
     </row>
     <row r="17" ht="23" customHeight="1">
@@ -1327,37 +1318,37 @@
         <v>22</v>
       </c>
       <c r="B17" s="7">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="C17" s="7">
-        <v>46104</v>
+        <v>46082</v>
       </c>
       <c r="D17" s="7">
-        <v>46104</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>25</v>
+        <v>46132</v>
+      </c>
+      <c r="E17" s="7">
+        <v>46097</v>
       </c>
       <c r="F17" s="8">
-        <v>-35</v>
+        <v>-8</v>
       </c>
       <c r="G17" s="8">
-        <v>-10</v>
+        <v>-8</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="I17" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="K17" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="M17" s="6" t="s">
         <v>25</v>
@@ -1372,13 +1363,13 @@
         <v>25</v>
       </c>
       <c r="Q17" s="6" t="s">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="R17" s="6" t="s">
         <v>35</v>
       </c>
       <c r="S17" s="9">
-        <v>357.49</v>
+        <v>146.55</v>
       </c>
     </row>
     <row r="18" ht="23" customHeight="1">
@@ -1389,19 +1380,19 @@
         <v>46132</v>
       </c>
       <c r="C18" s="7">
-        <v>46118</v>
+        <v>46132</v>
       </c>
       <c r="D18" s="7">
-        <v>46118</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>25</v>
+        <v>46132</v>
+      </c>
+      <c r="E18" s="7">
+        <v>46119</v>
       </c>
       <c r="F18" s="8">
-        <v>-21</v>
+        <v>-8</v>
       </c>
       <c r="G18" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>23</v>
@@ -1410,16 +1401,16 @@
         <v>23</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="K18" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="M18" s="6" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="N18" s="6" t="s">
         <v>27</v>
@@ -1428,16 +1419,16 @@
         <v>27</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="Q18" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="R18" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="S18" s="9">
-        <v>91.54</v>
+        <v>620</v>
       </c>
     </row>
     <row r="19" ht="23" customHeight="1">
@@ -1448,19 +1439,19 @@
         <v>46132</v>
       </c>
       <c r="C19" s="7">
-        <v>46082</v>
+        <v>46132</v>
       </c>
       <c r="D19" s="7">
         <v>46132</v>
       </c>
       <c r="E19" s="7">
-        <v>46097</v>
+        <v>46118</v>
       </c>
       <c r="F19" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G19" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>23</v>
@@ -1469,13 +1460,13 @@
         <v>23</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K19" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="M19" s="6" t="s">
         <v>25</v>
@@ -1490,13 +1481,13 @@
         <v>25</v>
       </c>
       <c r="Q19" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="R19" s="6" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="S19" s="9">
-        <v>146.55</v>
+        <v>620</v>
       </c>
     </row>
     <row r="20" ht="23" customHeight="1">
@@ -1507,19 +1498,19 @@
         <v>46132</v>
       </c>
       <c r="C20" s="7">
-        <v>46118</v>
+        <v>46132</v>
       </c>
       <c r="D20" s="7">
-        <v>46118</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>25</v>
+        <v>46132</v>
+      </c>
+      <c r="E20" s="7">
+        <v>46086</v>
       </c>
       <c r="F20" s="8">
-        <v>-21</v>
+        <v>-8</v>
       </c>
       <c r="G20" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>23</v>
@@ -1534,10 +1525,10 @@
         <v>25</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="M20" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N20" s="6" t="s">
         <v>27</v>
@@ -1549,13 +1540,13 @@
         <v>25</v>
       </c>
       <c r="Q20" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="R20" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S20" s="9">
-        <v>200</v>
+        <v>620</v>
       </c>
     </row>
     <row r="21" ht="23" customHeight="1">
@@ -1566,35 +1557,35 @@
         <v>46132</v>
       </c>
       <c r="C21" s="7">
-        <v>45901</v>
+        <v>46132</v>
       </c>
       <c r="D21" s="7">
-        <v>45938</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>25</v>
+        <v>46132</v>
+      </c>
+      <c r="E21" s="7">
+        <v>46057</v>
       </c>
       <c r="F21" s="8">
-        <v>-201</v>
+        <v>-8</v>
       </c>
       <c r="G21" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H21" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L21" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="I21" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J21" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="K21" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L21" s="6" t="s">
-        <v>60</v>
-      </c>
       <c r="M21" s="6" t="s">
         <v>25</v>
       </c>
@@ -1608,13 +1599,13 @@
         <v>25</v>
       </c>
       <c r="Q21" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="R21" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S21" s="9">
-        <v>546</v>
+        <v>650</v>
       </c>
     </row>
     <row r="22" ht="23" customHeight="1">
@@ -1634,10 +1625,10 @@
         <v>46119</v>
       </c>
       <c r="F22" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G22" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H22" s="6" t="s">
         <v>23</v>
@@ -1646,16 +1637,16 @@
         <v>23</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="K22" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M22" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N22" s="6" t="s">
         <v>27</v>
@@ -1670,10 +1661,10 @@
         <v>28</v>
       </c>
       <c r="R22" s="6" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="S22" s="9">
-        <v>620</v>
+        <v>650</v>
       </c>
     </row>
     <row r="23" ht="23" customHeight="1">
@@ -1693,10 +1684,10 @@
         <v>46118</v>
       </c>
       <c r="F23" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G23" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H23" s="6" t="s">
         <v>23</v>
@@ -1705,13 +1696,13 @@
         <v>23</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K23" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="M23" s="6" t="s">
         <v>25</v>
@@ -1732,7 +1723,7 @@
         <v>29</v>
       </c>
       <c r="S23" s="9">
-        <v>620</v>
+        <v>680</v>
       </c>
     </row>
     <row r="24" ht="23" customHeight="1">
@@ -1749,13 +1740,13 @@
         <v>46132</v>
       </c>
       <c r="E24" s="7">
-        <v>46086</v>
+        <v>46113</v>
       </c>
       <c r="F24" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G24" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>23</v>
@@ -1764,16 +1755,16 @@
         <v>23</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="K24" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L24" s="6" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="M24" s="6" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="N24" s="6" t="s">
         <v>27</v>
@@ -1791,7 +1782,7 @@
         <v>29</v>
       </c>
       <c r="S24" s="9">
-        <v>620</v>
+        <v>680</v>
       </c>
     </row>
     <row r="25" ht="23" customHeight="1">
@@ -1808,13 +1799,13 @@
         <v>46132</v>
       </c>
       <c r="E25" s="7">
-        <v>46112</v>
+        <v>46087</v>
       </c>
       <c r="F25" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G25" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>23</v>
@@ -1823,13 +1814,13 @@
         <v>23</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K25" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L25" s="6" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="M25" s="6" t="s">
         <v>25</v>
@@ -1850,7 +1841,7 @@
         <v>29</v>
       </c>
       <c r="S25" s="9">
-        <v>630</v>
+        <v>680</v>
       </c>
     </row>
     <row r="26" ht="23" customHeight="1">
@@ -1858,19 +1849,19 @@
         <v>22</v>
       </c>
       <c r="B26" s="7">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="C26" s="7">
-        <v>46132</v>
+        <v>46118</v>
       </c>
       <c r="D26" s="7">
-        <v>46132</v>
-      </c>
-      <c r="E26" s="7">
-        <v>46119</v>
+        <v>46111</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F26" s="8">
-        <v>-7</v>
+        <v>-29</v>
       </c>
       <c r="G26" s="8">
         <v>-7</v>
@@ -1882,16 +1873,16 @@
         <v>23</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="K26" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L26" s="6" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="M26" s="6" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="N26" s="6" t="s">
         <v>27</v>
@@ -1903,13 +1894,13 @@
         <v>25</v>
       </c>
       <c r="Q26" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="R26" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="S26" s="9">
-        <v>650</v>
+        <v>321.17</v>
       </c>
     </row>
     <row r="27" ht="23" customHeight="1">
@@ -1917,16 +1908,16 @@
         <v>22</v>
       </c>
       <c r="B27" s="7">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="C27" s="7">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="D27" s="7">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="E27" s="7">
-        <v>46057</v>
+        <v>46100</v>
       </c>
       <c r="F27" s="8">
         <v>-7</v>
@@ -1941,13 +1932,13 @@
         <v>23</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="K27" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L27" s="6" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="M27" s="6" t="s">
         <v>25</v>
@@ -1965,10 +1956,10 @@
         <v>28</v>
       </c>
       <c r="R27" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="S27" s="9">
-        <v>650</v>
+        <v>680</v>
       </c>
     </row>
     <row r="28" ht="23" customHeight="1">
@@ -1976,22 +1967,22 @@
         <v>22</v>
       </c>
       <c r="B28" s="7">
-        <v>46132</v>
+        <v>46134</v>
       </c>
       <c r="C28" s="7">
-        <v>46132</v>
+        <v>46082</v>
       </c>
       <c r="D28" s="7">
-        <v>46132</v>
-      </c>
-      <c r="E28" s="7">
-        <v>46087</v>
+        <v>46125</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F28" s="8">
-        <v>-7</v>
+        <v>-15</v>
       </c>
       <c r="G28" s="8">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="H28" s="6" t="s">
         <v>23</v>
@@ -2000,13 +1991,13 @@
         <v>23</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="K28" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L28" s="6" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="M28" s="6" t="s">
         <v>25</v>
@@ -2021,13 +2012,13 @@
         <v>25</v>
       </c>
       <c r="Q28" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="R28" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="S28" s="9">
-        <v>680</v>
+        <v>79.05</v>
       </c>
     </row>
     <row r="29" ht="23" customHeight="1">
@@ -2035,7 +2026,7 @@
         <v>22</v>
       </c>
       <c r="B29" s="7">
-        <v>46132</v>
+        <v>46134</v>
       </c>
       <c r="C29" s="7">
         <v>46132</v>
@@ -2043,14 +2034,14 @@
       <c r="D29" s="7">
         <v>46132</v>
       </c>
-      <c r="E29" s="7">
-        <v>46118</v>
+      <c r="E29" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F29" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G29" s="8">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="H29" s="6" t="s">
         <v>23</v>
@@ -2059,16 +2050,16 @@
         <v>23</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K29" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L29" s="6" t="s">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="M29" s="6" t="s">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="N29" s="6" t="s">
         <v>27</v>
@@ -2080,13 +2071,13 @@
         <v>25</v>
       </c>
       <c r="Q29" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="R29" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S29" s="9">
-        <v>680</v>
+        <v>200</v>
       </c>
     </row>
     <row r="30" ht="23" customHeight="1">
@@ -2094,22 +2085,22 @@
         <v>22</v>
       </c>
       <c r="B30" s="7">
-        <v>46132</v>
+        <v>46135</v>
       </c>
       <c r="C30" s="7">
-        <v>46132</v>
+        <v>46125</v>
       </c>
       <c r="D30" s="7">
-        <v>46132</v>
-      </c>
-      <c r="E30" s="7">
-        <v>46113</v>
+        <v>46125</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F30" s="8">
-        <v>-7</v>
+        <v>-15</v>
       </c>
       <c r="G30" s="8">
-        <v>-7</v>
+        <v>-5</v>
       </c>
       <c r="H30" s="6" t="s">
         <v>23</v>
@@ -2118,16 +2109,16 @@
         <v>23</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K30" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L30" s="6" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="M30" s="6" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="N30" s="6" t="s">
         <v>27</v>
@@ -2139,13 +2130,13 @@
         <v>25</v>
       </c>
       <c r="Q30" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="R30" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S30" s="9">
-        <v>680</v>
+        <v>550</v>
       </c>
     </row>
     <row r="31" ht="23" customHeight="1">
@@ -2153,22 +2144,22 @@
         <v>22</v>
       </c>
       <c r="B31" s="7">
-        <v>46133</v>
+        <v>46135</v>
       </c>
       <c r="C31" s="7">
-        <v>46118</v>
+        <v>46132</v>
       </c>
       <c r="D31" s="7">
-        <v>46111</v>
+        <v>46132</v>
       </c>
       <c r="E31" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F31" s="8">
-        <v>-28</v>
+        <v>-8</v>
       </c>
       <c r="G31" s="8">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="H31" s="6" t="s">
         <v>23</v>
@@ -2177,34 +2168,34 @@
         <v>23</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="K31" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L31" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="M31" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="N31" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O31" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P31" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="M31" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="N31" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="O31" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="P31" s="6" t="s">
-        <v>25</v>
-      </c>
       <c r="Q31" s="6" t="s">
         <v>25</v>
       </c>
       <c r="R31" s="6" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="S31" s="9">
-        <v>321.17</v>
+        <v>650</v>
       </c>
     </row>
     <row r="32" ht="23" customHeight="1">
@@ -2212,22 +2203,22 @@
         <v>22</v>
       </c>
       <c r="B32" s="7">
-        <v>46133</v>
+        <v>46136</v>
       </c>
       <c r="C32" s="7">
-        <v>46133</v>
+        <v>46118</v>
       </c>
       <c r="D32" s="7">
-        <v>46133</v>
-      </c>
-      <c r="E32" s="7">
-        <v>46100</v>
+        <v>46118</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F32" s="8">
-        <v>-6</v>
+        <v>-22</v>
       </c>
       <c r="G32" s="8">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="H32" s="6" t="s">
         <v>23</v>
@@ -2236,13 +2227,13 @@
         <v>23</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K32" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L32" s="6" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="M32" s="6" t="s">
         <v>25</v>
@@ -2257,13 +2248,13 @@
         <v>25</v>
       </c>
       <c r="Q32" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="R32" s="6" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="S32" s="9">
-        <v>680</v>
+        <v>100</v>
       </c>
     </row>
     <row r="33" ht="23" customHeight="1">
@@ -2271,22 +2262,22 @@
         <v>22</v>
       </c>
       <c r="B33" s="7">
-        <v>46134</v>
+        <v>46136</v>
       </c>
       <c r="C33" s="7">
-        <v>46082</v>
+        <v>46111</v>
       </c>
       <c r="D33" s="7">
-        <v>46125</v>
+        <v>46111</v>
       </c>
       <c r="E33" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F33" s="8">
-        <v>-14</v>
+        <v>-29</v>
       </c>
       <c r="G33" s="8">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="H33" s="6" t="s">
         <v>23</v>
@@ -2295,13 +2286,13 @@
         <v>23</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="K33" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L33" s="6" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="M33" s="6" t="s">
         <v>25</v>
@@ -2319,10 +2310,10 @@
         <v>25</v>
       </c>
       <c r="R33" s="6" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="S33" s="9">
-        <v>79.05</v>
+        <v>180</v>
       </c>
     </row>
     <row r="34" ht="23" customHeight="1">
@@ -2330,22 +2321,22 @@
         <v>22</v>
       </c>
       <c r="B34" s="7">
-        <v>46134</v>
+        <v>46136</v>
       </c>
       <c r="C34" s="7">
-        <v>46132</v>
+        <v>46125</v>
       </c>
       <c r="D34" s="7">
-        <v>46132</v>
+        <v>46125</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F34" s="8">
-        <v>-7</v>
+        <v>-15</v>
       </c>
       <c r="G34" s="8">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="H34" s="6" t="s">
         <v>23</v>
@@ -2354,16 +2345,16 @@
         <v>23</v>
       </c>
       <c r="J34" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L34" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="K34" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L34" s="6" t="s">
-        <v>76</v>
-      </c>
       <c r="M34" s="6" t="s">
-        <v>76</v>
+        <v>25</v>
       </c>
       <c r="N34" s="6" t="s">
         <v>27</v>
@@ -2381,7 +2372,7 @@
         <v>29</v>
       </c>
       <c r="S34" s="9">
-        <v>200</v>
+        <v>302.72</v>
       </c>
     </row>
     <row r="35" ht="23" customHeight="1">
@@ -2389,22 +2380,22 @@
         <v>22</v>
       </c>
       <c r="B35" s="7">
-        <v>46134</v>
+        <v>46139</v>
       </c>
       <c r="C35" s="7">
-        <v>46132</v>
+        <v>46082</v>
       </c>
       <c r="D35" s="7">
-        <v>46132</v>
-      </c>
-      <c r="E35" s="7" t="s">
-        <v>25</v>
+        <v>46139</v>
+      </c>
+      <c r="E35" s="7">
+        <v>46097</v>
       </c>
       <c r="F35" s="8">
-        <v>-7</v>
+        <v>-1</v>
       </c>
       <c r="G35" s="8">
-        <v>-5</v>
+        <v>-1</v>
       </c>
       <c r="H35" s="6" t="s">
         <v>23</v>
@@ -2413,13 +2404,13 @@
         <v>23</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="K35" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L35" s="6" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="M35" s="6" t="s">
         <v>25</v>
@@ -2434,13 +2425,13 @@
         <v>25</v>
       </c>
       <c r="Q35" s="6" t="s">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="R35" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="S35" s="9">
-        <v>200</v>
+        <v>146.55</v>
       </c>
     </row>
     <row r="36" ht="23" customHeight="1">
@@ -2448,37 +2439,37 @@
         <v>22</v>
       </c>
       <c r="B36" s="7">
-        <v>46135</v>
+        <v>46139</v>
       </c>
       <c r="C36" s="7">
-        <v>46125</v>
+        <v>46111</v>
       </c>
       <c r="D36" s="7">
-        <v>46125</v>
+        <v>46083</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F36" s="8">
-        <v>-14</v>
+        <v>-57</v>
       </c>
       <c r="G36" s="8">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="I36" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="K36" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L36" s="6" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="M36" s="6" t="s">
         <v>25</v>
@@ -2499,7 +2490,7 @@
         <v>29</v>
       </c>
       <c r="S36" s="9">
-        <v>550</v>
+        <v>320</v>
       </c>
     </row>
     <row r="37" ht="23" customHeight="1">
@@ -2507,38 +2498,38 @@
         <v>22</v>
       </c>
       <c r="B37" s="7">
-        <v>46135</v>
+        <v>46139</v>
       </c>
       <c r="C37" s="7">
-        <v>46132</v>
+        <v>45901</v>
       </c>
       <c r="D37" s="7">
-        <v>46132</v>
+        <v>45938</v>
       </c>
       <c r="E37" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F37" s="8">
-        <v>-7</v>
+        <v>-202</v>
       </c>
       <c r="G37" s="8">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
       <c r="I37" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J37" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L37" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="K37" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L37" s="6" t="s">
-        <v>80</v>
-      </c>
       <c r="M37" s="6" t="s">
         <v>25</v>
       </c>
@@ -2549,7 +2540,7 @@
         <v>27</v>
       </c>
       <c r="P37" s="6" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="Q37" s="6" t="s">
         <v>25</v>
@@ -2558,7 +2549,7 @@
         <v>29</v>
       </c>
       <c r="S37" s="9">
-        <v>650</v>
+        <v>426</v>
       </c>
     </row>
     <row r="38" ht="23" customHeight="1">
@@ -2566,22 +2557,22 @@
         <v>22</v>
       </c>
       <c r="B38" s="7">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="C38" s="7">
-        <v>46111</v>
+        <v>46132</v>
       </c>
       <c r="D38" s="7">
-        <v>46111</v>
+        <v>46132</v>
       </c>
       <c r="E38" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F38" s="8">
-        <v>-28</v>
+        <v>-8</v>
       </c>
       <c r="G38" s="8">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="H38" s="6" t="s">
         <v>23</v>
@@ -2590,13 +2581,13 @@
         <v>23</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K38" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="M38" s="6" t="s">
         <v>25</v>
@@ -2617,7 +2608,7 @@
         <v>29</v>
       </c>
       <c r="S38" s="9">
-        <v>180</v>
+        <v>500</v>
       </c>
     </row>
     <row r="39" ht="23" customHeight="1">
@@ -2625,22 +2616,22 @@
         <v>22</v>
       </c>
       <c r="B39" s="7">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="C39" s="7">
-        <v>46125</v>
+        <v>46139</v>
       </c>
       <c r="D39" s="7">
-        <v>46125</v>
-      </c>
-      <c r="E39" s="7" t="s">
-        <v>25</v>
+        <v>46139</v>
+      </c>
+      <c r="E39" s="7">
+        <v>46127</v>
       </c>
       <c r="F39" s="8">
-        <v>-14</v>
+        <v>-1</v>
       </c>
       <c r="G39" s="8">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="H39" s="6" t="s">
         <v>23</v>
@@ -2649,16 +2640,16 @@
         <v>23</v>
       </c>
       <c r="J39" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="K39" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L39" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="K39" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L39" s="6" t="s">
-        <v>66</v>
-      </c>
       <c r="M39" s="6" t="s">
-        <v>25</v>
+        <v>82</v>
       </c>
       <c r="N39" s="6" t="s">
         <v>27</v>
@@ -2670,13 +2661,13 @@
         <v>25</v>
       </c>
       <c r="Q39" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="R39" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S39" s="9">
-        <v>302.72</v>
+        <v>600</v>
       </c>
     </row>
     <row r="40" ht="23" customHeight="1">
@@ -2687,55 +2678,55 @@
         <v>46139</v>
       </c>
       <c r="C40" s="7">
-        <v>46082</v>
+        <v>46139</v>
       </c>
       <c r="D40" s="7">
         <v>46139</v>
       </c>
       <c r="E40" s="7">
-        <v>46097</v>
+        <v>46119</v>
       </c>
       <c r="F40" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G40" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I40" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>54</v>
+        <v>83</v>
       </c>
       <c r="K40" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L40" s="6" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="M40" s="6" t="s">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P40" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q40" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="R40" s="6" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="S40" s="9">
-        <v>146.55</v>
+        <v>600</v>
       </c>
     </row>
     <row r="41" ht="23" customHeight="1">
@@ -2746,25 +2737,25 @@
         <v>46139</v>
       </c>
       <c r="C41" s="7">
-        <v>46111</v>
+        <v>46139</v>
       </c>
       <c r="D41" s="7">
-        <v>46083</v>
-      </c>
-      <c r="E41" s="7" t="s">
-        <v>25</v>
+        <v>46139</v>
+      </c>
+      <c r="E41" s="7">
+        <v>46112</v>
       </c>
       <c r="F41" s="8">
-        <v>-56</v>
+        <v>-1</v>
       </c>
       <c r="G41" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J41" s="6" t="s">
         <v>84</v>
@@ -2773,28 +2764,28 @@
         <v>25</v>
       </c>
       <c r="L41" s="6" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="M41" s="6" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="N41" s="6" t="s">
         <v>27</v>
       </c>
       <c r="O41" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P41" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q41" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="R41" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S41" s="9">
-        <v>320</v>
+        <v>600</v>
       </c>
     </row>
     <row r="42" ht="23" customHeight="1">
@@ -2808,22 +2799,22 @@
         <v>46139</v>
       </c>
       <c r="D42" s="7">
-        <v>46139</v>
+        <v>46104</v>
       </c>
       <c r="E42" s="7">
-        <v>46119</v>
+        <v>46057</v>
       </c>
       <c r="F42" s="8">
-        <v>0</v>
+        <v>-36</v>
       </c>
       <c r="G42" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="I42" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J42" s="6" t="s">
         <v>85</v>
@@ -2832,16 +2823,16 @@
         <v>25</v>
       </c>
       <c r="L42" s="6" t="s">
-        <v>76</v>
+        <v>44</v>
       </c>
       <c r="M42" s="6" t="s">
-        <v>76</v>
+        <v>25</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>25</v>
@@ -2853,7 +2844,7 @@
         <v>29</v>
       </c>
       <c r="S42" s="9">
-        <v>600</v>
+        <v>620</v>
       </c>
     </row>
     <row r="43" ht="23" customHeight="1">
@@ -2870,19 +2861,19 @@
         <v>46139</v>
       </c>
       <c r="E43" s="7">
-        <v>46112</v>
+        <v>46119</v>
       </c>
       <c r="F43" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G43" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I43" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J43" s="6" t="s">
         <v>86</v>
@@ -2891,16 +2882,16 @@
         <v>25</v>
       </c>
       <c r="L43" s="6" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="M43" s="6" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O43" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P43" s="6" t="s">
         <v>25</v>
@@ -2909,10 +2900,10 @@
         <v>28</v>
       </c>
       <c r="R43" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="S43" s="9">
-        <v>600</v>
+        <v>620</v>
       </c>
     </row>
     <row r="44" ht="23" customHeight="1">
@@ -2932,16 +2923,16 @@
         <v>46127</v>
       </c>
       <c r="F44" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G44" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I44" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J44" s="6" t="s">
         <v>87</v>
@@ -2953,13 +2944,13 @@
         <v>88</v>
       </c>
       <c r="M44" s="6" t="s">
-        <v>88</v>
+        <v>25</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P44" s="6" t="s">
         <v>25</v>
@@ -2971,7 +2962,7 @@
         <v>29</v>
       </c>
       <c r="S44" s="9">
-        <v>600</v>
+        <v>630</v>
       </c>
     </row>
     <row r="45" ht="23" customHeight="1">
@@ -2988,19 +2979,19 @@
         <v>46139</v>
       </c>
       <c r="E45" s="7">
-        <v>46119</v>
+        <v>46100</v>
       </c>
       <c r="F45" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G45" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J45" s="6" t="s">
         <v>89</v>
@@ -3009,16 +3000,16 @@
         <v>25</v>
       </c>
       <c r="L45" s="6" t="s">
-        <v>62</v>
+        <v>90</v>
       </c>
       <c r="M45" s="6" t="s">
-        <v>62</v>
+        <v>25</v>
       </c>
       <c r="N45" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O45" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P45" s="6" t="s">
         <v>25</v>
@@ -3027,10 +3018,10 @@
         <v>28</v>
       </c>
       <c r="R45" s="6" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="S45" s="9">
-        <v>620</v>
+        <v>630</v>
       </c>
     </row>
     <row r="46" ht="23" customHeight="1">
@@ -3044,31 +3035,31 @@
         <v>46139</v>
       </c>
       <c r="D46" s="7">
-        <v>46104</v>
+        <v>46139</v>
       </c>
       <c r="E46" s="7">
-        <v>46057</v>
+        <v>46100</v>
       </c>
       <c r="F46" s="8">
-        <v>-35</v>
+        <v>-1</v>
       </c>
       <c r="G46" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K46" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L46" s="6" t="s">
-        <v>46</v>
+        <v>79</v>
       </c>
       <c r="M46" s="6" t="s">
         <v>25</v>
@@ -3077,7 +3068,7 @@
         <v>27</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>25</v>
@@ -3089,7 +3080,7 @@
         <v>29</v>
       </c>
       <c r="S46" s="9">
-        <v>620</v>
+        <v>630</v>
       </c>
     </row>
     <row r="47" ht="23" customHeight="1">
@@ -3109,34 +3100,34 @@
         <v>46112</v>
       </c>
       <c r="F47" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G47" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J47" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K47" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L47" s="6" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="M47" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N47" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O47" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P47" s="6" t="s">
         <v>25</v>
@@ -3165,37 +3156,37 @@
         <v>46139</v>
       </c>
       <c r="E48" s="7">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="F48" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G48" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J48" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K48" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L48" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="M48" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P48" s="6" t="s">
         <v>25</v>
@@ -3224,40 +3215,40 @@
         <v>46139</v>
       </c>
       <c r="E49" s="7">
-        <v>46100</v>
+        <v>46119</v>
       </c>
       <c r="F49" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G49" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="K49" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>60</v>
+        <v>96</v>
       </c>
       <c r="M49" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N49" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O49" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P49" s="6" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="Q49" s="6" t="s">
         <v>28</v>
@@ -3283,37 +3274,37 @@
         <v>46139</v>
       </c>
       <c r="E50" s="7">
-        <v>46112</v>
+        <v>46119</v>
       </c>
       <c r="F50" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G50" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I50" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J50" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="K50" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L50" s="6" t="s">
-        <v>96</v>
+        <v>60</v>
       </c>
       <c r="M50" s="6" t="s">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P50" s="6" t="s">
         <v>25</v>
@@ -3325,7 +3316,7 @@
         <v>29</v>
       </c>
       <c r="S50" s="9">
-        <v>630</v>
+        <v>650</v>
       </c>
     </row>
     <row r="51" ht="23" customHeight="1">
@@ -3339,43 +3330,43 @@
         <v>46139</v>
       </c>
       <c r="D51" s="7">
-        <v>46139</v>
+        <v>46104</v>
       </c>
       <c r="E51" s="7">
-        <v>46119</v>
+        <v>46057</v>
       </c>
       <c r="F51" s="8">
-        <v>0</v>
+        <v>-36</v>
       </c>
       <c r="G51" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K51" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L51" s="6" t="s">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="M51" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N51" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O51" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P51" s="6" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="Q51" s="6" t="s">
         <v>28</v>
@@ -3384,7 +3375,7 @@
         <v>29</v>
       </c>
       <c r="S51" s="9">
-        <v>630</v>
+        <v>650</v>
       </c>
     </row>
     <row r="52" ht="23" customHeight="1">
@@ -3401,19 +3392,19 @@
         <v>46139</v>
       </c>
       <c r="E52" s="7">
-        <v>46127</v>
+        <v>46101</v>
       </c>
       <c r="F52" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G52" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J52" s="6" t="s">
         <v>99</v>
@@ -3428,10 +3419,10 @@
         <v>25</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P52" s="6" t="s">
         <v>25</v>
@@ -3443,7 +3434,7 @@
         <v>29</v>
       </c>
       <c r="S52" s="9">
-        <v>630</v>
+        <v>650</v>
       </c>
     </row>
     <row r="53" ht="23" customHeight="1">
@@ -3463,16 +3454,16 @@
         <v>46127</v>
       </c>
       <c r="F53" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G53" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J53" s="6" t="s">
         <v>101</v>
@@ -3487,10 +3478,10 @@
         <v>25</v>
       </c>
       <c r="N53" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O53" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P53" s="6" t="s">
         <v>25</v>
@@ -3522,16 +3513,16 @@
         <v>46122</v>
       </c>
       <c r="F54" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G54" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H54" s="6" t="s">
         <v>23</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J54" s="6" t="s">
         <v>103</v>
@@ -3549,7 +3540,7 @@
         <v>27</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P54" s="6" t="s">
         <v>25</v>
@@ -3581,16 +3572,16 @@
         <v>46119</v>
       </c>
       <c r="F55" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G55" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J55" s="6" t="s">
         <v>104</v>
@@ -3599,16 +3590,16 @@
         <v>25</v>
       </c>
       <c r="L55" s="6" t="s">
-        <v>37</v>
+        <v>105</v>
       </c>
       <c r="M55" s="6" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="N55" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O55" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P55" s="6" t="s">
         <v>25</v>
@@ -3620,7 +3611,7 @@
         <v>29</v>
       </c>
       <c r="S55" s="9">
-        <v>650</v>
+        <v>670</v>
       </c>
     </row>
     <row r="56" ht="23" customHeight="1">
@@ -3637,37 +3628,37 @@
         <v>46139</v>
       </c>
       <c r="E56" s="7">
-        <v>46101</v>
+        <v>46119</v>
       </c>
       <c r="F56" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G56" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J56" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K56" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L56" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M56" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P56" s="6" t="s">
         <v>25</v>
@@ -3679,7 +3670,7 @@
         <v>29</v>
       </c>
       <c r="S56" s="9">
-        <v>650</v>
+        <v>680</v>
       </c>
     </row>
     <row r="57" ht="23" customHeight="1">
@@ -3693,40 +3684,40 @@
         <v>46139</v>
       </c>
       <c r="D57" s="7">
-        <v>46104</v>
+        <v>46139</v>
       </c>
       <c r="E57" s="7">
-        <v>46057</v>
+        <v>46113</v>
       </c>
       <c r="F57" s="8">
-        <v>-35</v>
+        <v>-1</v>
       </c>
       <c r="G57" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="I57" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J57" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K57" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L57" s="6" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="M57" s="6" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="N57" s="6" t="s">
         <v>27</v>
       </c>
       <c r="O57" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P57" s="6" t="s">
         <v>25</v>
@@ -3738,7 +3729,7 @@
         <v>29</v>
       </c>
       <c r="S57" s="9">
-        <v>650</v>
+        <v>680</v>
       </c>
     </row>
     <row r="58" ht="23" customHeight="1">
@@ -3755,37 +3746,37 @@
         <v>46139</v>
       </c>
       <c r="E58" s="7">
-        <v>46092</v>
+        <v>46100</v>
       </c>
       <c r="F58" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G58" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I58" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J58" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K58" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L58" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="M58" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P58" s="6" t="s">
         <v>25</v>
@@ -3797,7 +3788,7 @@
         <v>29</v>
       </c>
       <c r="S58" s="9">
-        <v>650</v>
+        <v>680</v>
       </c>
     </row>
     <row r="59" ht="23" customHeight="1">
@@ -3814,40 +3805,40 @@
         <v>46139</v>
       </c>
       <c r="E59" s="7">
-        <v>46119</v>
+        <v>46127</v>
       </c>
       <c r="F59" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G59" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I59" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J59" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K59" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L59" s="6" t="s">
-        <v>111</v>
+        <v>49</v>
       </c>
       <c r="M59" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N59" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O59" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P59" s="6" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="Q59" s="6" t="s">
         <v>28</v>
@@ -3856,7 +3847,7 @@
         <v>29</v>
       </c>
       <c r="S59" s="9">
-        <v>670</v>
+        <v>680</v>
       </c>
     </row>
     <row r="60" ht="23" customHeight="1">
@@ -3876,16 +3867,16 @@
         <v>46119</v>
       </c>
       <c r="F60" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G60" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I60" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J60" s="6" t="s">
         <v>112</v>
@@ -3894,16 +3885,16 @@
         <v>25</v>
       </c>
       <c r="L60" s="6" t="s">
-        <v>113</v>
+        <v>47</v>
       </c>
       <c r="M60" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P60" s="6" t="s">
         <v>25</v>
@@ -3912,7 +3903,7 @@
         <v>28</v>
       </c>
       <c r="R60" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="S60" s="9">
         <v>680</v>
@@ -3932,37 +3923,37 @@
         <v>46139</v>
       </c>
       <c r="E61" s="7">
-        <v>46113</v>
+        <v>46099</v>
       </c>
       <c r="F61" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G61" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I61" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J61" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="K61" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L61" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="K61" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L61" s="6" t="s">
-        <v>42</v>
-      </c>
       <c r="M61" s="6" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="N61" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O61" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P61" s="6" t="s">
         <v>25</v>
@@ -3971,10 +3962,10 @@
         <v>28</v>
       </c>
       <c r="R61" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="S61" s="9">
-        <v>680</v>
+        <v>700</v>
       </c>
     </row>
     <row r="62" ht="23" customHeight="1">
@@ -3991,19 +3982,19 @@
         <v>46139</v>
       </c>
       <c r="E62" s="7">
-        <v>46100</v>
+        <v>46092</v>
       </c>
       <c r="F62" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G62" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I62" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J62" s="6" t="s">
         <v>115</v>
@@ -4018,10 +4009,10 @@
         <v>25</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P62" s="6" t="s">
         <v>25</v>
@@ -4033,7 +4024,7 @@
         <v>29</v>
       </c>
       <c r="S62" s="9">
-        <v>680</v>
+        <v>700</v>
       </c>
     </row>
     <row r="63" ht="23" customHeight="1">
@@ -4053,16 +4044,16 @@
         <v>46119</v>
       </c>
       <c r="F63" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G63" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I63" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J63" s="6" t="s">
         <v>117</v>
@@ -4071,28 +4062,28 @@
         <v>25</v>
       </c>
       <c r="L63" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="M63" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="N63" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O63" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P63" s="6" t="s">
         <v>50</v>
-      </c>
-      <c r="M63" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="N63" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="O63" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="P63" s="6" t="s">
-        <v>25</v>
       </c>
       <c r="Q63" s="6" t="s">
         <v>28</v>
       </c>
       <c r="R63" s="6" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="S63" s="9">
-        <v>680</v>
+        <v>700</v>
       </c>
     </row>
     <row r="64" ht="23" customHeight="1">
@@ -4109,19 +4100,19 @@
         <v>46139</v>
       </c>
       <c r="E64" s="7">
-        <v>46127</v>
+        <v>46129</v>
       </c>
       <c r="F64" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G64" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I64" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J64" s="6" t="s">
         <v>118</v>
@@ -4130,28 +4121,28 @@
         <v>25</v>
       </c>
       <c r="L64" s="6" t="s">
-        <v>52</v>
+        <v>119</v>
       </c>
       <c r="M64" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="P64" s="6" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="Q64" s="6" t="s">
         <v>28</v>
       </c>
       <c r="R64" s="6" t="s">
-        <v>29</v>
+        <v>120</v>
       </c>
       <c r="S64" s="9">
-        <v>680</v>
+        <v>800</v>
       </c>
     </row>
     <row r="65" ht="23" customHeight="1">
@@ -4159,58 +4150,58 @@
         <v>22</v>
       </c>
       <c r="B65" s="7">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="C65" s="7">
-        <v>46139</v>
+        <v>46132</v>
       </c>
       <c r="D65" s="7">
-        <v>46139</v>
-      </c>
-      <c r="E65" s="7">
-        <v>46099</v>
+        <v>46132</v>
+      </c>
+      <c r="E65" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F65" s="8">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="G65" s="8">
         <v>0</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I65" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J65" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="K65" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L65" s="6" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="M65" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N65" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O65" s="6" t="s">
-        <v>83</v>
+        <v>122</v>
       </c>
       <c r="P65" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q65" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="R65" s="6" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="S65" s="9">
-        <v>700</v>
+        <v>110.69</v>
       </c>
     </row>
     <row r="66" ht="23" customHeight="1">
@@ -4218,7 +4209,7 @@
         <v>22</v>
       </c>
       <c r="B66" s="7">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="C66" s="7">
         <v>46139</v>
@@ -4226,50 +4217,50 @@
       <c r="D66" s="7">
         <v>46139</v>
       </c>
-      <c r="E66" s="7">
-        <v>46092</v>
+      <c r="E66" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F66" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G66" s="8">
         <v>0</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I66" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J66" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="K66" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L66" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="M66" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="N66" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O66" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="M66" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="N66" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="O66" s="6" t="s">
-        <v>83</v>
-      </c>
       <c r="P66" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q66" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="R66" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S66" s="9">
-        <v>700</v>
+        <v>120</v>
       </c>
     </row>
     <row r="67" ht="23" customHeight="1">
@@ -4277,58 +4268,58 @@
         <v>22</v>
       </c>
       <c r="B67" s="7">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="C67" s="7">
-        <v>46139</v>
+        <v>46132</v>
       </c>
       <c r="D67" s="7">
-        <v>46139</v>
-      </c>
-      <c r="E67" s="7">
-        <v>46119</v>
+        <v>46132</v>
+      </c>
+      <c r="E67" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F67" s="8">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="G67" s="8">
         <v>0</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I67" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J67" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="K67" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L67" s="6" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="M67" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N67" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O67" s="6" t="s">
-        <v>83</v>
+        <v>122</v>
       </c>
       <c r="P67" s="6" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="Q67" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="R67" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S67" s="9">
-        <v>700</v>
+        <v>124.25</v>
       </c>
     </row>
     <row r="68" ht="23" customHeight="1">
@@ -4336,58 +4327,58 @@
         <v>22</v>
       </c>
       <c r="B68" s="7">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="C68" s="7">
-        <v>46139</v>
+        <v>46125</v>
       </c>
       <c r="D68" s="7">
-        <v>46139</v>
-      </c>
-      <c r="E68" s="7">
-        <v>46129</v>
+        <v>46125</v>
+      </c>
+      <c r="E68" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F68" s="8">
-        <v>0</v>
+        <v>-15</v>
       </c>
       <c r="G68" s="8">
         <v>0</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I68" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J68" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="K68" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L68" s="6" t="s">
-        <v>125</v>
+        <v>47</v>
       </c>
       <c r="M68" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>83</v>
+        <v>122</v>
       </c>
       <c r="P68" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q68" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="R68" s="6" t="s">
-        <v>126</v>
+        <v>35</v>
       </c>
       <c r="S68" s="9">
-        <v>800</v>
+        <v>408.24</v>
       </c>
     </row>
     <row r="69" ht="23" customHeight="1">
@@ -4398,22 +4389,22 @@
         <v>46140</v>
       </c>
       <c r="C69" s="7">
-        <v>46132</v>
+        <v>46140</v>
       </c>
       <c r="D69" s="7">
-        <v>46132</v>
-      </c>
-      <c r="E69" s="7" t="s">
-        <v>25</v>
+        <v>46140</v>
+      </c>
+      <c r="E69" s="7">
+        <v>46100</v>
       </c>
       <c r="F69" s="8">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="G69" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I69" s="6" t="s">
         <v>25</v>
@@ -4425,28 +4416,28 @@
         <v>25</v>
       </c>
       <c r="L69" s="6" t="s">
-        <v>116</v>
+        <v>66</v>
       </c>
       <c r="M69" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>27</v>
+        <v>122</v>
       </c>
       <c r="O69" s="6" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="P69" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q69" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="R69" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="S69" s="9">
-        <v>110.69</v>
+        <v>680</v>
       </c>
     </row>
     <row r="70" ht="23" customHeight="1">
@@ -4454,46 +4445,46 @@
         <v>22</v>
       </c>
       <c r="B70" s="7">
-        <v>46140</v>
+        <v>46142</v>
       </c>
       <c r="C70" s="7">
-        <v>46132</v>
+        <v>45930</v>
       </c>
       <c r="D70" s="7">
-        <v>46132</v>
+        <v>46142</v>
       </c>
       <c r="E70" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F70" s="8">
-        <v>-7</v>
+        <v>2</v>
       </c>
       <c r="G70" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I70" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J70" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K70" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L70" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="M70" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="N70" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="K70" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L70" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="M70" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="N70" s="6" t="s">
-        <v>27</v>
-      </c>
       <c r="O70" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P70" s="6" t="s">
         <v>25</v>
@@ -4502,246 +4493,69 @@
         <v>25</v>
       </c>
       <c r="R70" s="6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="S70" s="9">
-        <v>124.25</v>
+        <v>185.5</v>
       </c>
     </row>
     <row r="71" ht="23" customHeight="1">
-      <c r="A71" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B71" s="7">
-        <v>46140</v>
-      </c>
-      <c r="C71" s="7">
-        <v>46125</v>
-      </c>
-      <c r="D71" s="7">
-        <v>46125</v>
-      </c>
-      <c r="E71" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F71" s="8">
-        <v>-14</v>
-      </c>
-      <c r="G71" s="8">
-        <v>1</v>
-      </c>
-      <c r="H71" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I71" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="J71" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="K71" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L71" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="M71" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="N71" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="O71" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="P71" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q71" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="R71" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="S71" s="9">
-        <v>408.24</v>
-      </c>
-    </row>
-    <row r="72" ht="23" customHeight="1">
-      <c r="A72" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B72" s="7">
-        <v>46140</v>
-      </c>
-      <c r="C72" s="7">
-        <v>46140</v>
-      </c>
-      <c r="D72" s="7">
-        <v>46140</v>
-      </c>
-      <c r="E72" s="7">
-        <v>46100</v>
-      </c>
-      <c r="F72" s="8">
-        <v>1</v>
-      </c>
-      <c r="G72" s="8">
-        <v>1</v>
-      </c>
-      <c r="H72" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="I72" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="J72" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="K72" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L72" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="M72" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="N72" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="O72" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="P72" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q72" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="R72" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="S72" s="9">
-        <v>680</v>
-      </c>
-    </row>
-    <row r="73" ht="23" customHeight="1">
-      <c r="A73" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B73" s="7">
-        <v>46142</v>
-      </c>
-      <c r="C73" s="7">
-        <v>45930</v>
-      </c>
-      <c r="D73" s="7">
-        <v>46142</v>
-      </c>
-      <c r="E73" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F73" s="8">
-        <v>3</v>
-      </c>
-      <c r="G73" s="8">
-        <v>3</v>
-      </c>
-      <c r="H73" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="I73" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="J73" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="K73" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L73" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="M73" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="N73" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="O73" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="P73" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q73" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="R73" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="S73" s="9">
-        <v>185.5</v>
-      </c>
-    </row>
-    <row r="74" ht="23" customHeight="1">
-      <c r="A74" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B74" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C74" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="D74" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="E74" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="F74" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="G74" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="H74" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="I74" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="J74" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="K74" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="L74" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="M74" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="N74" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="O74" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="P74" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q74" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="R74" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="S74" s="13">
-        <f>SUM(S6:S73)</f>
+      <c r="A71" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B71" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C71" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D71" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E71" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F71" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="G71" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="H71" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="I71" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="J71" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="K71" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="L71" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="M71" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="N71" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="O71" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="P71" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q71" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="R71" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="S71" s="13">
+        <f>SUM(S6:S70)</f>
       </c>
     </row>
   </sheetData>

</xml_diff>